<commit_message>
Reconciled data models.datasets on WinEventLog & XmlWinEventLog
</commit_message>
<xml_diff>
--- a/cim_sourcetype_inventory.xlsx
+++ b/cim_sourcetype_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JamesHBaxter\Dropbox\Programming\splunk-cim-reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0787D7E-A02C-43F5-B7DC-6C8E578D50E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7E3DAE7-2855-47E1-A1CE-7F3DC12964CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28125" yWindow="2820" windowWidth="23400" windowHeight="19185" xr2:uid="{9B46642C-0618-4BD2-A18B-2F59CC5C4C41}"/>
+    <workbookView xWindow="-27615" yWindow="3330" windowWidth="23400" windowHeight="19185" xr2:uid="{9B46642C-0618-4BD2-A18B-2F59CC5C4C41}"/>
   </bookViews>
   <sheets>
     <sheet name="cim_sourcetype_inventory" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7816" uniqueCount="2772">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7816" uniqueCount="2771">
   <si>
     <t>sourcetype</t>
   </si>
@@ -7993,9 +7993,6 @@
     <t>WinEventLog</t>
   </si>
   <si>
-    <t>Authentication.Authentication, Endpoint.Processes, Malware.Malware_Operations</t>
-  </si>
-  <si>
     <t>Windows Event Log</t>
   </si>
   <si>
@@ -8197,9 +8194,6 @@
     <t>XmlWinEventLog</t>
   </si>
   <si>
-    <t>Authentication.Authentication, Change.All_Changes, Endpoint.Processes, Intrusion_Detection.IDS_Attacks, Updates.Updates</t>
-  </si>
-  <si>
     <t>Windows XML Event Logs</t>
   </si>
   <si>
@@ -8339,6 +8333,9 @@
   </si>
   <si>
     <t>openSUSE / SLES zypper package manager log from /var/log/zypp/history - install/update/remove transactions on SUSE-family hosts.</t>
+  </si>
+  <si>
+    <t>Authentication.Authentication, Change.All_Changes, Endpoint.Ports, Endpoint.Processes, Endpoint.Registry, Endpoint.Services, Intrusion_Detection.IDS_Attacks, Malware.Malware_Operations, Updates.Updates</t>
   </si>
 </sst>
 </file>
@@ -33233,16 +33230,16 @@
         <v>35</v>
       </c>
       <c r="F810" t="s">
-        <v>2656</v>
+        <v>2770</v>
       </c>
       <c r="G810" t="s">
         <v>37</v>
       </c>
       <c r="H810" t="s">
+        <v>2656</v>
+      </c>
+      <c r="I810" t="s">
         <v>2657</v>
-      </c>
-      <c r="I810" t="s">
-        <v>2658</v>
       </c>
       <c r="J810" t="s">
         <v>19</v>
@@ -33250,7 +33247,7 @@
     </row>
     <row r="811" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A811" t="s">
-        <v>2659</v>
+        <v>2658</v>
       </c>
       <c r="B811" t="s">
         <v>34</v>
@@ -33268,10 +33265,10 @@
         <v>37</v>
       </c>
       <c r="H811" t="s">
+        <v>2659</v>
+      </c>
+      <c r="I811" t="s">
         <v>2660</v>
-      </c>
-      <c r="I811" t="s">
-        <v>2661</v>
       </c>
       <c r="J811" t="s">
         <v>19</v>
@@ -33279,7 +33276,7 @@
     </row>
     <row r="812" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A812" t="s">
-        <v>2662</v>
+        <v>2661</v>
       </c>
       <c r="B812" t="s">
         <v>34</v>
@@ -33300,10 +33297,10 @@
         <v>37</v>
       </c>
       <c r="H812" t="s">
+        <v>2662</v>
+      </c>
+      <c r="I812" t="s">
         <v>2663</v>
-      </c>
-      <c r="I812" t="s">
-        <v>2664</v>
       </c>
       <c r="J812" t="s">
         <v>19</v>
@@ -33311,7 +33308,7 @@
     </row>
     <row r="813" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A813" t="s">
-        <v>2665</v>
+        <v>2664</v>
       </c>
       <c r="B813" t="s">
         <v>34</v>
@@ -33329,10 +33326,10 @@
         <v>37</v>
       </c>
       <c r="H813" t="s">
+        <v>2665</v>
+      </c>
+      <c r="I813" t="s">
         <v>2666</v>
-      </c>
-      <c r="I813" t="s">
-        <v>2667</v>
       </c>
       <c r="J813" t="s">
         <v>19</v>
@@ -33340,7 +33337,7 @@
     </row>
     <row r="814" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A814" t="s">
-        <v>2668</v>
+        <v>2667</v>
       </c>
       <c r="B814" t="s">
         <v>34</v>
@@ -33361,10 +33358,10 @@
         <v>37</v>
       </c>
       <c r="H814" t="s">
+        <v>2668</v>
+      </c>
+      <c r="I814" t="s">
         <v>2669</v>
-      </c>
-      <c r="I814" t="s">
-        <v>2670</v>
       </c>
       <c r="J814" t="s">
         <v>19</v>
@@ -33372,7 +33369,7 @@
     </row>
     <row r="815" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A815" t="s">
-        <v>2671</v>
+        <v>2670</v>
       </c>
       <c r="B815" t="s">
         <v>34</v>
@@ -33393,10 +33390,10 @@
         <v>37</v>
       </c>
       <c r="H815" t="s">
+        <v>2671</v>
+      </c>
+      <c r="I815" t="s">
         <v>2672</v>
-      </c>
-      <c r="I815" t="s">
-        <v>2673</v>
       </c>
       <c r="J815" t="s">
         <v>19</v>
@@ -33404,7 +33401,7 @@
     </row>
     <row r="816" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A816" t="s">
-        <v>2674</v>
+        <v>2673</v>
       </c>
       <c r="B816" t="s">
         <v>34</v>
@@ -33425,10 +33422,10 @@
         <v>37</v>
       </c>
       <c r="H816" t="s">
+        <v>2674</v>
+      </c>
+      <c r="I816" t="s">
         <v>2675</v>
-      </c>
-      <c r="I816" t="s">
-        <v>2676</v>
       </c>
       <c r="J816" t="s">
         <v>19</v>
@@ -33436,7 +33433,7 @@
     </row>
     <row r="817" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A817" t="s">
-        <v>2677</v>
+        <v>2676</v>
       </c>
       <c r="B817" t="s">
         <v>34</v>
@@ -33457,10 +33454,10 @@
         <v>37</v>
       </c>
       <c r="H817" t="s">
+        <v>2677</v>
+      </c>
+      <c r="I817" t="s">
         <v>2678</v>
-      </c>
-      <c r="I817" t="s">
-        <v>2679</v>
       </c>
       <c r="J817" t="s">
         <v>19</v>
@@ -33468,7 +33465,7 @@
     </row>
     <row r="818" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A818" t="s">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="B818" t="s">
         <v>34</v>
@@ -33489,10 +33486,10 @@
         <v>37</v>
       </c>
       <c r="H818" t="s">
+        <v>2680</v>
+      </c>
+      <c r="I818" t="s">
         <v>2681</v>
-      </c>
-      <c r="I818" t="s">
-        <v>2682</v>
       </c>
       <c r="J818" t="s">
         <v>19</v>
@@ -33500,7 +33497,7 @@
     </row>
     <row r="819" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A819" t="s">
-        <v>2683</v>
+        <v>2682</v>
       </c>
       <c r="B819" t="s">
         <v>34</v>
@@ -33521,10 +33518,10 @@
         <v>37</v>
       </c>
       <c r="H819" t="s">
+        <v>2683</v>
+      </c>
+      <c r="I819" t="s">
         <v>2684</v>
-      </c>
-      <c r="I819" t="s">
-        <v>2685</v>
       </c>
       <c r="J819" t="s">
         <v>19</v>
@@ -33532,7 +33529,7 @@
     </row>
     <row r="820" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A820" t="s">
-        <v>2686</v>
+        <v>2685</v>
       </c>
       <c r="B820" t="s">
         <v>34</v>
@@ -33553,10 +33550,10 @@
         <v>37</v>
       </c>
       <c r="H820" t="s">
+        <v>2686</v>
+      </c>
+      <c r="I820" t="s">
         <v>2687</v>
-      </c>
-      <c r="I820" t="s">
-        <v>2688</v>
       </c>
       <c r="J820" t="s">
         <v>19</v>
@@ -33564,7 +33561,7 @@
     </row>
     <row r="821" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A821" t="s">
-        <v>2689</v>
+        <v>2688</v>
       </c>
       <c r="B821" t="s">
         <v>34</v>
@@ -33579,16 +33576,16 @@
         <v>35</v>
       </c>
       <c r="F821" t="s">
-        <v>2690</v>
+        <v>2689</v>
       </c>
       <c r="G821" t="s">
         <v>37</v>
       </c>
       <c r="H821" t="s">
+        <v>2690</v>
+      </c>
+      <c r="I821" t="s">
         <v>2691</v>
-      </c>
-      <c r="I821" t="s">
-        <v>2692</v>
       </c>
       <c r="J821" t="s">
         <v>19</v>
@@ -33596,7 +33593,7 @@
     </row>
     <row r="822" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A822" t="s">
-        <v>2693</v>
+        <v>2692</v>
       </c>
       <c r="B822" t="s">
         <v>34</v>
@@ -33617,10 +33614,10 @@
         <v>37</v>
       </c>
       <c r="H822" t="s">
+        <v>2693</v>
+      </c>
+      <c r="I822" t="s">
         <v>2694</v>
-      </c>
-      <c r="I822" t="s">
-        <v>2695</v>
       </c>
       <c r="J822" t="s">
         <v>19</v>
@@ -33628,7 +33625,7 @@
     </row>
     <row r="823" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A823" t="s">
-        <v>2696</v>
+        <v>2695</v>
       </c>
       <c r="B823" t="s">
         <v>34</v>
@@ -33649,10 +33646,10 @@
         <v>37</v>
       </c>
       <c r="H823" t="s">
+        <v>2696</v>
+      </c>
+      <c r="I823" t="s">
         <v>2697</v>
-      </c>
-      <c r="I823" t="s">
-        <v>2698</v>
       </c>
       <c r="J823" t="s">
         <v>19</v>
@@ -33660,7 +33657,7 @@
     </row>
     <row r="824" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A824" t="s">
-        <v>2699</v>
+        <v>2698</v>
       </c>
       <c r="B824" t="s">
         <v>34</v>
@@ -33681,10 +33678,10 @@
         <v>37</v>
       </c>
       <c r="H824" t="s">
+        <v>2699</v>
+      </c>
+      <c r="I824" t="s">
         <v>2700</v>
-      </c>
-      <c r="I824" t="s">
-        <v>2701</v>
       </c>
       <c r="J824" t="s">
         <v>19</v>
@@ -33692,7 +33689,7 @@
     </row>
     <row r="825" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A825" t="s">
-        <v>2702</v>
+        <v>2701</v>
       </c>
       <c r="B825" t="s">
         <v>34</v>
@@ -33713,10 +33710,10 @@
         <v>37</v>
       </c>
       <c r="H825" t="s">
+        <v>2702</v>
+      </c>
+      <c r="I825" t="s">
         <v>2703</v>
-      </c>
-      <c r="I825" t="s">
-        <v>2704</v>
       </c>
       <c r="J825" t="s">
         <v>19</v>
@@ -33724,7 +33721,7 @@
     </row>
     <row r="826" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A826" t="s">
-        <v>2705</v>
+        <v>2704</v>
       </c>
       <c r="B826" t="s">
         <v>34</v>
@@ -33745,10 +33742,10 @@
         <v>37</v>
       </c>
       <c r="H826" t="s">
+        <v>2705</v>
+      </c>
+      <c r="I826" t="s">
         <v>2706</v>
-      </c>
-      <c r="I826" t="s">
-        <v>2707</v>
       </c>
       <c r="J826" t="s">
         <v>19</v>
@@ -33756,7 +33753,7 @@
     </row>
     <row r="827" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A827" t="s">
-        <v>2708</v>
+        <v>2707</v>
       </c>
       <c r="B827" t="s">
         <v>34</v>
@@ -33774,10 +33771,10 @@
         <v>37</v>
       </c>
       <c r="H827" t="s">
+        <v>2708</v>
+      </c>
+      <c r="I827" t="s">
         <v>2709</v>
-      </c>
-      <c r="I827" t="s">
-        <v>2710</v>
       </c>
       <c r="J827" t="s">
         <v>19</v>
@@ -33785,7 +33782,7 @@
     </row>
     <row r="828" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A828" t="s">
-        <v>2711</v>
+        <v>2710</v>
       </c>
       <c r="B828" t="s">
         <v>34</v>
@@ -33803,10 +33800,10 @@
         <v>37</v>
       </c>
       <c r="H828" t="s">
+        <v>2711</v>
+      </c>
+      <c r="I828" t="s">
         <v>2712</v>
-      </c>
-      <c r="I828" t="s">
-        <v>2713</v>
       </c>
       <c r="J828" t="s">
         <v>19</v>
@@ -33814,7 +33811,7 @@
     </row>
     <row r="829" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A829" t="s">
-        <v>2714</v>
+        <v>2713</v>
       </c>
       <c r="B829" t="s">
         <v>169</v>
@@ -33832,10 +33829,10 @@
         <v>2541</v>
       </c>
       <c r="H829" t="s">
+        <v>2714</v>
+      </c>
+      <c r="I829" t="s">
         <v>2715</v>
-      </c>
-      <c r="I829" t="s">
-        <v>2716</v>
       </c>
       <c r="J829" t="s">
         <v>19</v>
@@ -33843,7 +33840,7 @@
     </row>
     <row r="830" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A830" t="s">
-        <v>2717</v>
+        <v>2716</v>
       </c>
       <c r="B830" t="s">
         <v>11</v>
@@ -33861,10 +33858,10 @@
         <v>84</v>
       </c>
       <c r="H830" t="s">
+        <v>2717</v>
+      </c>
+      <c r="I830" t="s">
         <v>2718</v>
-      </c>
-      <c r="I830" t="s">
-        <v>2719</v>
       </c>
       <c r="J830" t="s">
         <v>19</v>
@@ -33872,7 +33869,7 @@
     </row>
     <row r="831" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A831" t="s">
-        <v>2720</v>
+        <v>2719</v>
       </c>
       <c r="B831" t="s">
         <v>34</v>
@@ -33890,10 +33887,10 @@
         <v>37</v>
       </c>
       <c r="H831" t="s">
+        <v>2720</v>
+      </c>
+      <c r="I831" t="s">
         <v>2721</v>
-      </c>
-      <c r="I831" t="s">
-        <v>2722</v>
       </c>
       <c r="J831" t="s">
         <v>19</v>
@@ -33901,7 +33898,7 @@
     </row>
     <row r="832" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A832" t="s">
-        <v>2723</v>
+        <v>2722</v>
       </c>
       <c r="B832" t="s">
         <v>34</v>
@@ -33916,16 +33913,16 @@
         <v>35</v>
       </c>
       <c r="F832" t="s">
-        <v>2724</v>
+        <v>2770</v>
       </c>
       <c r="G832" t="s">
         <v>37</v>
       </c>
       <c r="H832" t="s">
-        <v>2725</v>
+        <v>2723</v>
       </c>
       <c r="I832" t="s">
-        <v>2726</v>
+        <v>2724</v>
       </c>
       <c r="J832" t="s">
         <v>19</v>
@@ -33933,7 +33930,7 @@
     </row>
     <row r="833" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A833" t="s">
-        <v>2727</v>
+        <v>2725</v>
       </c>
       <c r="B833" t="s">
         <v>34</v>
@@ -33948,16 +33945,16 @@
         <v>35</v>
       </c>
       <c r="F833" t="s">
-        <v>2728</v>
+        <v>2726</v>
       </c>
       <c r="G833" t="s">
         <v>37</v>
       </c>
       <c r="H833" t="s">
-        <v>2729</v>
+        <v>2727</v>
       </c>
       <c r="I833" t="s">
-        <v>2730</v>
+        <v>2728</v>
       </c>
       <c r="J833" t="s">
         <v>19</v>
@@ -33965,7 +33962,7 @@
     </row>
     <row r="834" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A834" t="s">
-        <v>2731</v>
+        <v>2729</v>
       </c>
       <c r="B834" t="s">
         <v>34</v>
@@ -33988,7 +33985,7 @@
     </row>
     <row r="835" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A835" t="s">
-        <v>2732</v>
+        <v>2730</v>
       </c>
       <c r="B835" t="s">
         <v>34</v>
@@ -33999,7 +33996,7 @@
     </row>
     <row r="836" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A836" t="s">
-        <v>2733</v>
+        <v>2731</v>
       </c>
       <c r="B836" t="s">
         <v>34</v>
@@ -34010,7 +34007,7 @@
     </row>
     <row r="837" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A837" t="s">
-        <v>2734</v>
+        <v>2732</v>
       </c>
       <c r="B837" t="s">
         <v>34</v>
@@ -34021,7 +34018,7 @@
     </row>
     <row r="838" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A838" t="s">
-        <v>2735</v>
+        <v>2733</v>
       </c>
       <c r="B838" t="s">
         <v>34</v>
@@ -34035,7 +34032,7 @@
     </row>
     <row r="839" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A839" t="s">
-        <v>2736</v>
+        <v>2734</v>
       </c>
       <c r="B839" t="s">
         <v>34</v>
@@ -34055,7 +34052,7 @@
     </row>
     <row r="840" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A840" t="s">
-        <v>2737</v>
+        <v>2735</v>
       </c>
       <c r="B840" t="s">
         <v>34</v>
@@ -34066,7 +34063,7 @@
     </row>
     <row r="841" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A841" t="s">
-        <v>2738</v>
+        <v>2736</v>
       </c>
       <c r="B841" t="s">
         <v>11</v>
@@ -34081,10 +34078,10 @@
         <v>84</v>
       </c>
       <c r="H841" t="s">
-        <v>2739</v>
+        <v>2737</v>
       </c>
       <c r="I841" t="s">
-        <v>2740</v>
+        <v>2738</v>
       </c>
       <c r="J841" t="s">
         <v>19</v>
@@ -34092,7 +34089,7 @@
     </row>
     <row r="842" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A842" t="s">
-        <v>2741</v>
+        <v>2739</v>
       </c>
       <c r="B842" t="s">
         <v>12</v>
@@ -34113,10 +34110,10 @@
         <v>1227</v>
       </c>
       <c r="H842" t="s">
-        <v>2742</v>
+        <v>2740</v>
       </c>
       <c r="I842" t="s">
-        <v>2743</v>
+        <v>2741</v>
       </c>
       <c r="J842" t="s">
         <v>19</v>
@@ -34124,7 +34121,7 @@
     </row>
     <row r="843" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A843" t="s">
-        <v>2744</v>
+        <v>2742</v>
       </c>
       <c r="B843" t="s">
         <v>12</v>
@@ -34142,13 +34139,13 @@
         <v>15</v>
       </c>
       <c r="G843" t="s">
+        <v>2743</v>
+      </c>
+      <c r="H843" t="s">
+        <v>2744</v>
+      </c>
+      <c r="I843" t="s">
         <v>2745</v>
-      </c>
-      <c r="H843" t="s">
-        <v>2746</v>
-      </c>
-      <c r="I843" t="s">
-        <v>2747</v>
       </c>
       <c r="J843" t="s">
         <v>19</v>
@@ -34156,7 +34153,7 @@
     </row>
     <row r="844" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A844" t="s">
-        <v>2748</v>
+        <v>2746</v>
       </c>
       <c r="B844" t="s">
         <v>11</v>
@@ -34174,10 +34171,10 @@
         <v>84</v>
       </c>
       <c r="H844" t="s">
-        <v>2749</v>
+        <v>2747</v>
       </c>
       <c r="I844" t="s">
-        <v>2750</v>
+        <v>2748</v>
       </c>
       <c r="J844" t="s">
         <v>19</v>
@@ -34185,7 +34182,7 @@
     </row>
     <row r="845" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A845" t="s">
-        <v>2751</v>
+        <v>2749</v>
       </c>
       <c r="B845" t="s">
         <v>21</v>
@@ -34200,13 +34197,13 @@
         <v>899</v>
       </c>
       <c r="G845" t="s">
+        <v>2750</v>
+      </c>
+      <c r="H845" t="s">
+        <v>2751</v>
+      </c>
+      <c r="I845" t="s">
         <v>2752</v>
-      </c>
-      <c r="H845" t="s">
-        <v>2753</v>
-      </c>
-      <c r="I845" t="s">
-        <v>2754</v>
       </c>
       <c r="J845" t="s">
         <v>19</v>
@@ -34214,7 +34211,7 @@
     </row>
     <row r="846" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A846" t="s">
-        <v>2755</v>
+        <v>2753</v>
       </c>
       <c r="B846" t="s">
         <v>169</v>
@@ -34235,10 +34232,10 @@
         <v>615</v>
       </c>
       <c r="H846" t="s">
-        <v>2756</v>
+        <v>2754</v>
       </c>
       <c r="I846" t="s">
-        <v>2757</v>
+        <v>2755</v>
       </c>
       <c r="J846" t="s">
         <v>19</v>
@@ -34246,7 +34243,7 @@
     </row>
     <row r="847" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A847" t="s">
-        <v>2758</v>
+        <v>2756</v>
       </c>
       <c r="B847" t="s">
         <v>21</v>
@@ -34264,10 +34261,10 @@
         <v>23</v>
       </c>
       <c r="H847" t="s">
-        <v>2759</v>
+        <v>2757</v>
       </c>
       <c r="I847" t="s">
-        <v>2760</v>
+        <v>2758</v>
       </c>
       <c r="J847" t="s">
         <v>19</v>
@@ -34275,7 +34272,7 @@
     </row>
     <row r="848" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A848" t="s">
-        <v>2761</v>
+        <v>2759</v>
       </c>
       <c r="B848" t="s">
         <v>21</v>
@@ -34290,13 +34287,13 @@
         <v>15</v>
       </c>
       <c r="G848" t="s">
+        <v>2760</v>
+      </c>
+      <c r="H848" t="s">
+        <v>2761</v>
+      </c>
+      <c r="I848" t="s">
         <v>2762</v>
-      </c>
-      <c r="H848" t="s">
-        <v>2763</v>
-      </c>
-      <c r="I848" t="s">
-        <v>2764</v>
       </c>
       <c r="J848" t="s">
         <v>19</v>
@@ -34304,7 +34301,7 @@
     </row>
     <row r="849" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A849" t="s">
-        <v>2765</v>
+        <v>2763</v>
       </c>
       <c r="B849" t="s">
         <v>169</v>
@@ -34322,13 +34319,13 @@
         <v>602</v>
       </c>
       <c r="G849" t="s">
+        <v>2764</v>
+      </c>
+      <c r="H849" t="s">
+        <v>2765</v>
+      </c>
+      <c r="I849" t="s">
         <v>2766</v>
-      </c>
-      <c r="H849" t="s">
-        <v>2767</v>
-      </c>
-      <c r="I849" t="s">
-        <v>2768</v>
       </c>
       <c r="J849" t="s">
         <v>19</v>
@@ -34336,7 +34333,7 @@
     </row>
     <row r="850" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A850" t="s">
-        <v>2769</v>
+        <v>2767</v>
       </c>
       <c r="B850" t="s">
         <v>11</v>
@@ -34354,10 +34351,10 @@
         <v>84</v>
       </c>
       <c r="H850" t="s">
-        <v>2770</v>
+        <v>2768</v>
       </c>
       <c r="I850" t="s">
-        <v>2771</v>
+        <v>2769</v>
       </c>
       <c r="J850" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Updated CodeIntegrity/Operational from Malware to Change
</commit_message>
<xml_diff>
--- a/cim_sourcetype_inventory.xlsx
+++ b/cim_sourcetype_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JamesHBaxter\Dropbox\Programming\splunk-cim-reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7E3DAE7-2855-47E1-A1CE-7F3DC12964CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD060941-8AFB-4AA5-AD38-6E14B849EDAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27615" yWindow="3330" windowWidth="23400" windowHeight="19185" xr2:uid="{9B46642C-0618-4BD2-A18B-2F59CC5C4C41}"/>
+    <workbookView xWindow="-28125" yWindow="2820" windowWidth="23400" windowHeight="19185" xr2:uid="{9B46642C-0618-4BD2-A18B-2F59CC5C4C41}"/>
   </bookViews>
   <sheets>
     <sheet name="cim_sourcetype_inventory" sheetId="1" r:id="rId1"/>
@@ -33448,7 +33448,7 @@
         <v>35</v>
       </c>
       <c r="F817" t="s">
-        <v>196</v>
+        <v>43</v>
       </c>
       <c r="G817" t="s">
         <v>37</v>

</xml_diff>